<commit_message>
Reset Password Button Added
</commit_message>
<xml_diff>
--- a/Excel/students.xlsx
+++ b/Excel/students.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Jugal\College\Attendance_WELL\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91CAE724-A5A8-4C46-B1D7-2558C5843645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2588EDBF-23A3-421F-9EAC-C6731D1318B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{81B1BAD1-E213-4784-8BDE-9AD04D8DC3A3}"/>
+    <workbookView xWindow="3260" yWindow="3260" windowWidth="19200" windowHeight="11170" xr2:uid="{81B1BAD1-E213-4784-8BDE-9AD04D8DC3A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="138">
   <si>
     <t>password</t>
   </si>
@@ -60,12 +60,6 @@
     <t>student</t>
   </si>
   <si>
-    <t>Shail R. Shah</t>
-  </si>
-  <si>
-    <t>Jimit Patel</t>
-  </si>
-  <si>
     <t>Aagam Hiten Sheth</t>
   </si>
   <si>
@@ -129,9 +123,6 @@
     <t>Parth Pravinbhai Thakkar</t>
   </si>
   <si>
-    <t>Shayan Saiyed</t>
-  </si>
-  <si>
     <t>Shreyas Bhargavbhai Patel</t>
   </si>
   <si>
@@ -147,45 +138,6 @@
     <t>Vishwa Bhavin Chokshi</t>
   </si>
   <si>
-    <t>Lavina Tahliyani</t>
-  </si>
-  <si>
-    <t>Anant Kedia</t>
-  </si>
-  <si>
-    <t>Kevin Saurabh Mehta</t>
-  </si>
-  <si>
-    <t>Bhavya Sharma</t>
-  </si>
-  <si>
-    <t>Dhwani Acharya</t>
-  </si>
-  <si>
-    <t>Krisha Bhatt</t>
-  </si>
-  <si>
-    <t>Rakshith Jakinapally</t>
-  </si>
-  <si>
-    <t>Ritik Rakesh</t>
-  </si>
-  <si>
-    <t>Shree .</t>
-  </si>
-  <si>
-    <t>Vidhi Kothari</t>
-  </si>
-  <si>
-    <t>Vivek Maskar</t>
-  </si>
-  <si>
-    <t>AU2514030</t>
-  </si>
-  <si>
-    <t>AU2449005</t>
-  </si>
-  <si>
     <t>AU2544006</t>
   </si>
   <si>
@@ -249,9 +201,6 @@
     <t>AU2544017</t>
   </si>
   <si>
-    <t>AU2544023</t>
-  </si>
-  <si>
     <t>AU2544025</t>
   </si>
   <si>
@@ -267,45 +216,6 @@
     <t>AU2544019</t>
   </si>
   <si>
-    <t>AU2300053</t>
-  </si>
-  <si>
-    <t>AU2220040</t>
-  </si>
-  <si>
-    <t>AU2240116</t>
-  </si>
-  <si>
-    <t>AU24110006</t>
-  </si>
-  <si>
-    <t>AU24110005</t>
-  </si>
-  <si>
-    <t>AU24110002</t>
-  </si>
-  <si>
-    <t>AU24110015</t>
-  </si>
-  <si>
-    <t>AU24110010</t>
-  </si>
-  <si>
-    <t>AU24110008</t>
-  </si>
-  <si>
-    <t>AU24110007</t>
-  </si>
-  <si>
-    <t>AU24110011</t>
-  </si>
-  <si>
-    <t>shail.s@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>jimit.p@ahduni.edu.in</t>
-  </si>
-  <si>
     <t>aagam.s6@ahduni.edu.in</t>
   </si>
   <si>
@@ -369,9 +279,6 @@
     <t>parth.t2@ahduni.edu.in</t>
   </si>
   <si>
-    <t>shayan.s@ahduni.edu.in</t>
-  </si>
-  <si>
     <t>shreyas.p@ahduni.edu.in</t>
   </si>
   <si>
@@ -387,47 +294,167 @@
     <t>vishwa.c@ahduni.edu.in</t>
   </si>
   <si>
-    <t>lavina.t@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>anant.k@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>kevin.m1@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>bhavya.s12@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>dhwani.a@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>krisha.b2@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>rakshith.j@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>ritik.r@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>shree.s@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>vidhi.k3@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>vivek.m@ahduni.edu.in</t>
-  </si>
-  <si>
-    <t>CSE548 Applied Data Science</t>
+    <t>Nikita Arya</t>
+  </si>
+  <si>
+    <t>Nidhi Bosamiya</t>
+  </si>
+  <si>
+    <t>Patel Dhyey Sanjaybhai</t>
+  </si>
+  <si>
+    <t>Meet Bharat Rathi</t>
+  </si>
+  <si>
+    <t>Jayraj Derasari</t>
+  </si>
+  <si>
+    <t>Jay Raval</t>
+  </si>
+  <si>
+    <t>Dhruv Rakeshbhai Patel</t>
+  </si>
+  <si>
+    <t>Daksh Devalbhai Shah</t>
+  </si>
+  <si>
+    <t>Shalvi Anand Modi</t>
+  </si>
+  <si>
+    <t>Aneri Vimal Kabrawala</t>
+  </si>
+  <si>
+    <t>Aashi Sachin Shah</t>
+  </si>
+  <si>
+    <t>Aashaka Yagnesh Ashara</t>
+  </si>
+  <si>
+    <t>Yashvi Hitesh Modi</t>
+  </si>
+  <si>
+    <t>Kunjal Agarwal</t>
+  </si>
+  <si>
+    <t>Vrushti Yagneshbhai Patel</t>
+  </si>
+  <si>
+    <t>Yash Kirti</t>
+  </si>
+  <si>
+    <t>Diya Nagarbhai Patel</t>
+  </si>
+  <si>
+    <t>AU2220143</t>
+  </si>
+  <si>
+    <t>AU2449004</t>
+  </si>
+  <si>
+    <t>AU2240054</t>
+  </si>
+  <si>
+    <t>AU2240106</t>
+  </si>
+  <si>
+    <t>AU2240108</t>
+  </si>
+  <si>
+    <t>AU2240151</t>
+  </si>
+  <si>
+    <t>AU2240166</t>
+  </si>
+  <si>
+    <t>AU2240207</t>
+  </si>
+  <si>
+    <t>AU2240215</t>
+  </si>
+  <si>
+    <t>AU2340041</t>
+  </si>
+  <si>
+    <t>AU2340043</t>
+  </si>
+  <si>
+    <t>AU2340086</t>
+  </si>
+  <si>
+    <t>AU2340116</t>
+  </si>
+  <si>
+    <t>AU2340126</t>
+  </si>
+  <si>
+    <t>AU2340131</t>
+  </si>
+  <si>
+    <t>AU2340149</t>
+  </si>
+  <si>
+    <t>AU2340184</t>
+  </si>
+  <si>
+    <t>nikita.a1@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>nidhi.b2@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>dhyey.p5@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>meet.r@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>jayraj.d@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>jay.r1@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>dhruv.p6@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>daksh.s2@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>shalvi.m@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>aneri.k@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>aashi.s@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>aashaka.a@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>yashvi.m1@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>kunjal.a@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>vrushti.p@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>yash.k6@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>diya.p6@ahduni.edu.in</t>
+  </si>
+  <si>
+    <t>CSE602 Deep Learning</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -454,9 +481,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -491,24 +525,27 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{6BED7BF6-AD98-48FF-8502-4506D2846270}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{8E0185F9-59FB-40F5-A3EA-229B856DD28E}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -857,22 +894,22 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>8</v>
+        <v>86</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>48</v>
+        <v>103</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E2" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="6" t="s">
-        <v>128</v>
+      <c r="F2" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -880,22 +917,22 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>9</v>
+        <v>87</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>49</v>
+        <v>104</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>89</v>
+        <v>121</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E3" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>128</v>
+      <c r="F3" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -904,22 +941,22 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>128</v>
+      <c r="F4" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -928,22 +965,22 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E5" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>128</v>
+      <c r="F5" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -952,22 +989,22 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>52</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>128</v>
+      <c r="F6" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G6">
         <v>1</v>
@@ -976,22 +1013,22 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>93</v>
+        <v>60</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>128</v>
+      <c r="F7" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -1000,22 +1037,22 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>128</v>
+      <c r="F8" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -1024,22 +1061,22 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>128</v>
+      <c r="F9" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G9">
         <v>1</v>
@@ -1048,22 +1085,22 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="E10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>128</v>
+      <c r="F10" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G10">
         <v>1</v>
@@ -1071,22 +1108,22 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>128</v>
+      <c r="F11" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G11">
         <v>1</v>
@@ -1094,22 +1131,22 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F12" s="6" t="s">
-        <v>128</v>
+      <c r="F12" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G12">
         <v>1</v>
@@ -1117,22 +1154,22 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>128</v>
+      <c r="F13" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G13">
         <v>1</v>
@@ -1140,22 +1177,22 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="6" t="s">
-        <v>128</v>
+      <c r="F14" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G14">
         <v>1</v>
@@ -1163,22 +1200,22 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>128</v>
+      <c r="F15" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -1186,22 +1223,22 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>128</v>
+      <c r="F16" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -1209,22 +1246,22 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>103</v>
+        <v>70</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>128</v>
+      <c r="F17" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -1232,22 +1269,22 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E18" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>128</v>
+      <c r="F18" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -1255,22 +1292,22 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F19" s="6" t="s">
-        <v>128</v>
+      <c r="F19" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -1278,22 +1315,22 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>128</v>
+      <c r="F20" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G20">
         <v>1</v>
@@ -1301,22 +1338,22 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>107</v>
+        <v>66</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="6" t="s">
-        <v>128</v>
+      <c r="F21" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -1324,22 +1361,22 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E22" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>128</v>
+      <c r="F22" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -1347,22 +1384,22 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>109</v>
+        <v>63</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E23" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>128</v>
+      <c r="F23" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -1370,22 +1407,22 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="E24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>128</v>
+      <c r="F24" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -1393,22 +1430,22 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="E25" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F25" s="6" t="s">
-        <v>128</v>
+      <c r="F25" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -1416,22 +1453,22 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>112</v>
+        <v>65</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="E26" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E26" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>128</v>
+      <c r="F26" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G26">
         <v>1</v>
@@ -1439,22 +1476,22 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>73</v>
+        <v>41</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>113</v>
+        <v>67</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="E27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E27" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F27" s="6" t="s">
-        <v>128</v>
+      <c r="F27" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G27">
         <v>1</v>
@@ -1462,22 +1499,22 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>74</v>
+        <v>45</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E28" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>128</v>
+      <c r="F28" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G28">
         <v>1</v>
@@ -1485,22 +1522,22 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>115</v>
+        <v>68</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="E29" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E29" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F29" s="6" t="s">
-        <v>128</v>
+      <c r="F29" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G29">
         <v>1</v>
@@ -1508,22 +1545,22 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>36</v>
+        <v>88</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="E30" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E30" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>128</v>
+      <c r="F30" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G30">
         <v>1</v>
@@ -1531,22 +1568,22 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>37</v>
+        <v>89</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="E31" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E31" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F31" s="6" t="s">
-        <v>128</v>
+      <c r="F31" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G31">
         <v>1</v>
@@ -1554,22 +1591,22 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E32" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E32" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F32" s="6" t="s">
-        <v>128</v>
+      <c r="F32" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G32">
         <v>1</v>
@@ -1577,22 +1614,22 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>39</v>
+        <v>91</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>79</v>
+        <v>108</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="E33" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E33" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F33" s="6" t="s">
-        <v>128</v>
+      <c r="F33" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G33">
         <v>1</v>
@@ -1600,22 +1637,22 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>40</v>
+        <v>92</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E34" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E34" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F34" s="6" t="s">
-        <v>128</v>
+      <c r="F34" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G34">
         <v>1</v>
@@ -1623,22 +1660,22 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>41</v>
+        <v>93</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>81</v>
+        <v>110</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="E35" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F35" s="6" t="s">
-        <v>128</v>
+      <c r="F35" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G35">
         <v>1</v>
@@ -1646,22 +1683,22 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>42</v>
+        <v>94</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>82</v>
+        <v>111</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="E36" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E36" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F36" s="6" t="s">
-        <v>128</v>
+      <c r="F36" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G36">
         <v>1</v>
@@ -1669,22 +1706,22 @@
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>43</v>
+        <v>95</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>83</v>
+        <v>112</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E37" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F37" s="6" t="s">
-        <v>128</v>
+      <c r="F37" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G37">
         <v>1</v>
@@ -1692,22 +1729,22 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>44</v>
+        <v>96</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="E38" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E38" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F38" s="6" t="s">
-        <v>128</v>
+      <c r="F38" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G38">
         <v>1</v>
@@ -1715,22 +1752,22 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
-        <v>45</v>
+        <v>97</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E39" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E39" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>128</v>
+      <c r="F39" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G39">
         <v>1</v>
@@ -1738,22 +1775,22 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
-        <v>46</v>
+        <v>98</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="E40" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E40" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F40" s="6" t="s">
-        <v>128</v>
+      <c r="F40" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G40">
         <v>1</v>
@@ -1761,50 +1798,95 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>47</v>
+        <v>99</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="E41" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E41" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F41" s="6" t="s">
-        <v>128</v>
+      <c r="F41" s="7" t="s">
+        <v>137</v>
       </c>
       <c r="G41">
         <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="1"/>
+      <c r="A42" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="G42">
+        <v>1</v>
+      </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="1"/>
+      <c r="A43" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="G43">
+        <v>1</v>
+      </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="1"/>
+      <c r="A44" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="G44">
+        <v>1</v>
+      </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="2"/>

</xml_diff>